<commit_message>
fetch: sample-test-3docs -- 2026-07-17 20:54 UTC
</commit_message>
<xml_diff>
--- a/research-logs/fetch-log.xlsx
+++ b/research-logs/fetch-log.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,8 +42,18 @@
       <sz val="9"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001A5E38"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="007B3200"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +68,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD9B0"/>
       </patternFill>
     </fill>
   </fills>
@@ -101,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -113,6 +133,24 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -480,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1697,6 +1735,142 @@
       </c>
       <c r="J25" s="2" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="26" ht="55" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17 20:53:27 UTC</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>sample-test-3docs</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>[2606.00133] World Models: A Comprehensive Survey of Architectures, Methodologies, Reasoning Paradigms, and Applications</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2606.00133</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>798</v>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[2606.00133] World Models: A Comprehensive Survey of Architectures, Methodologies, Reasoning Paradigms, and Applications Skip to main content arXiv is now an independent nonprofit! Learn more × Search arXiv Press Enter to search · Advanced search Computer Science &gt; Machine Learning arXiv:2606.00133 </t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="27" ht="55" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17 20:53:27 UTC</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>sample-test-3docs</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Artificial</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>https://hai.stanford.edu/assets/files/ai_index_report_2026.pdf</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>16893</v>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence Index Report 2 0 2 6 AI INDEX REPORT 2026 Contents Introduction 2 Top Takeaways 9 1 Research and Development 12 2 Technical Performance 68 3 Responsible AI 126 4 Economy 171 5 Science 231 6 Medicine 255 7 Education 288 8 Policy and Governance 323 9 Public Opinion 360 Appendix</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="28" ht="55" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-17 20:53:38 UTC</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>sample-test-3docs</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>the state of ai</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>https://www.mckinsey.com/capabilities/quantumblack/our-insights/the-state-of-ai</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Timeout</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr"/>
+      <c r="G28" s="8" t="inlineStr"/>
+      <c r="H28" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="9" t="inlineStr">
+        <is>
+          <t>No response within 30s</t>
+        </is>
+      </c>
+      <c r="J28" s="8" t="n">
+        <v>30.14</v>
       </c>
     </row>
   </sheetData>
@@ -1725,6 +1899,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fetch: sample-test-v2 -- 2026-07-17 21:08 UTC
</commit_message>
<xml_diff>
--- a/research-logs/fetch-log.xlsx
+++ b/research-logs/fetch-log.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1871,6 +1871,142 @@
       </c>
       <c r="J28" s="8" t="n">
         <v>30.14</v>
+      </c>
+    </row>
+    <row r="29" ht="55" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:07:55 UTC</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>sample-test-v2</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>World Models: A Comprehensive Survey of Architectures, Methodologies, Reasoning Paradigms, and Applications</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2606.00133</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>PDF (arXiv abs-&gt;pdf rewrite (https://arxiv.org/abs/2606.00133))</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>28923</v>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>World Models: A Comprehensive Survey of Architectures, Methodologies, Reasoning Paradigms, and Applications Arif Hassan Zidan1, Yi Pan2, Hanqi Jiang2, Ruiyu Yan9, Wei Ruan2, Zihao Wu2, Lifeng Chen2, Weihang You2, Xinliang Li2, Bowen Chen3, Huawen Hu2, Peilong Wang10, Sizhuang Liu12, Jing Zhang5, Siy</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="n">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="30" ht="55" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:08:02 UTC</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>sample-test-v2</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Artificial</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>https://hai.stanford.edu/assets/files/ai_index_report_2026.pdf</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>16893</v>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence Index Report 2 0 2 6 AI INDEX REPORT 2026 Contents Introduction 2 Top Takeaways 9 1 Research and Development 12 2 Technical Performance 68 3 Responsible AI 126 4 Economy 171 5 Science 231 6 Medicine 255 7 Education 288 8 Policy and Governance 323 9 Public Opinion 360 Appendix</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="n">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="31" ht="55" customHeight="1">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:08:15 UTC</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>sample-test-v2</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>the state of ai</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>https://www.mckinsey.com/capabilities/quantumblack/our-insights/the-state-of-ai</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Timeout</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr"/>
+      <c r="G31" s="8" t="inlineStr"/>
+      <c r="H31" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="9" t="inlineStr">
+        <is>
+          <t>No response within 30s</t>
+        </is>
+      </c>
+      <c r="J31" s="8" t="n">
+        <v>30.06</v>
       </c>
     </row>
   </sheetData>
@@ -1902,6 +2038,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fetch: sample-test-v3 -- 2026-07-17 21:11 UTC
</commit_message>
<xml_diff>
--- a/research-logs/fetch-log.xlsx
+++ b/research-logs/fetch-log.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2006,6 +2006,142 @@
         </is>
       </c>
       <c r="J31" s="8" t="n">
+        <v>30.06</v>
+      </c>
+    </row>
+    <row r="32" ht="55" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:10:51 UTC</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>sample-test-v3</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>World Models: A Comprehensive Survey of Architectures, Methodologies, Reasoning Paradigms, and Applications</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2606.00133</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>PDF (arXiv abs-&gt;pdf rewrite (https://arxiv.org/abs/2606.00133))</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>19075</v>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>World Models: A Comprehensive Survey of Architectures, Methodologies, Reasoning Paradigms, and Applications Arif Hassan Zidan1, Yi Pan2, Hanqi Jiang2, Ruiyu Yan9, Wei Ruan2, Zihao Wu2, Lifeng Chen2, Weihang You2, Xinliang Li2, Bowen Chen3, Huawen Hu2, Peilong Wang10, Sizhuang Liu12, Jing Zhang5, Siy</t>
+        </is>
+      </c>
+      <c r="J32" s="5" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="33" ht="55" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:10:55 UTC</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>sample-test-v3</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Artificial</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>https://hai.stanford.edu/assets/files/ai_index_report_2026.pdf</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>3961</v>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence Index Report 2 0 2 6 AI INDEX REPORT 2026 Contents Introduction 2 Top Takeaways 9 1 Research and Development 12 2 Technical Performance 68 3 Responsible AI 126 4 Economy 171 5 Science 231 6 Medicine 255 7 Education 288 8 Policy and Governance 323 9 Public Opinion 360 Appendix</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="34" ht="55" customHeight="1">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:10:57 UTC</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>sample-test-v3</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>the state of ai</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>https://www.mckinsey.com/capabilities/quantumblack/our-insights/the-state-of-ai</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Timeout</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr"/>
+      <c r="G34" s="8" t="inlineStr"/>
+      <c r="H34" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="9" t="inlineStr">
+        <is>
+          <t>No response within 30s</t>
+        </is>
+      </c>
+      <c r="J34" s="8" t="n">
         <v>30.06</v>
       </c>
     </row>
@@ -2041,6 +2177,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fetch: full-source-test-24docs -- 2026-07-17 21:20 UTC
</commit_message>
<xml_diff>
--- a/research-logs/fetch-log.xlsx
+++ b/research-logs/fetch-log.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,8 +52,13 @@
       <color rgb="007B3200"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="007B4F00"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -78,6 +83,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFD9B0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -121,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -151,6 +161,15 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -518,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2143,6 +2162,1082 @@
       </c>
       <c r="J34" s="8" t="n">
         <v>30.06</v>
+      </c>
+    </row>
+    <row r="35" ht="55" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:19:25 UTC</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Artificial</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>https://hai.stanford.edu/assets/files/ai_index_report_2026.pdf</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>3961</v>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence Index Report 2 0 2 6 AI INDEX REPORT 2026 Contents Introduction 2 Top Takeaways 9 1 Research and Development 12 2 Technical Performance 68 3 Responsible AI 126 4 Economy 171 5 Science 231 6 Medicine 255 7 Education 288 8 Policy and Governance 323 9 Public Opinion 360 Appendix</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="36" ht="55" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:19:26 UTC</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>https://hai.stanford.edu/ai-index/2026</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="H36" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" s="12" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="J36" s="11" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="37" ht="55" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:19:26 UTC</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>NVIDIA in Brief</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>https://resources.nvidia.com/en-zz-ai-strategy/state-of-ai-2026</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>PDF (HTML-&gt;PDF link: https://www.nvidia.com/content/dam/en-zz/Solutions/about-nvidia/corporate-nvidia-in-brief.pdf)</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>705</v>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>N VIDIA in Brief NVIDIA pioneered accelerated computing. Today, our technology powers the world’s AI infrastructure, transforming every industry. Learn more. Company History Impact by Industry Founded in 1993, NVIDIA is the world leader in accelerated computing and AI. Automotive Our invention of th</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="n">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="38" ht="55" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:19:27 UTC</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>2026 06 cosmos 3 world foundation model</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>https://research.nvidia.com/publication/2026-06_cosmos-3-world-foundation-model</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="n">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="39" ht="55" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:19:28 UTC</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>genie 3</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>https://deepmind.google/research/publications/genie-3/</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="40" ht="55" customHeight="1">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:19:28 UTC</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>the state of ai</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>https://www.mckinsey.com/capabilities/quantumblack/our-insights/the-state-of-ai</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Timeout</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr"/>
+      <c r="G40" s="8" t="inlineStr"/>
+      <c r="H40" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="9" t="inlineStr">
+        <is>
+          <t>No response within 30s</t>
+        </is>
+      </c>
+      <c r="J40" s="8" t="n">
+        <v>30.12</v>
+      </c>
+    </row>
+    <row r="41" ht="55" customHeight="1">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:19:58 UTC</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>the state of ai shifting to the agentic era</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>https://www.mckinsey.com/capabilities/mckinsey-digital/our-insights/the-state-of-ai-shifting-to-the-agentic-era</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Timeout</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr"/>
+      <c r="G41" s="8" t="inlineStr"/>
+      <c r="H41" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="9" t="inlineStr">
+        <is>
+          <t>No response within 30s</t>
+        </is>
+      </c>
+      <c r="J41" s="8" t="n">
+        <v>30.18</v>
+      </c>
+    </row>
+    <row r="42" ht="55" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:28 UTC</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>hype cycle for agentic ai 2026</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>https://www.gartner.com/en/articles/hype-cycle-for-agentic-ai-2026</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>403</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="43" ht="55" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:28 UTC</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>ai agents reshape enterprise infrastructure 2026</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>https://www.gartner.com/en/documents/ai-agents-reshape-enterprise-infrastructure-2026</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>403</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="44" ht="55" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>ai infrastructure.html</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>https://www2.deloitte.com/us/en/insights/focus/tech-trends/2026/ai-infrastructure.html</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="45" ht="55" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Economics of AI | AI trends &amp; strategy | Oxford Economics</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>https://www.oxfordeconomics.com/resource/the-economics-of-ai/</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>2016</v>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>Economics of AI | AI trends &amp; strategy | Oxford Economics Skip to content Trending Topic The economics of AI Explore how AI is reshaping the global economy, from productivity and labour markets to investment, infrastructure, and risk. Contact us Featured Webinar AI and the economy: your questions an</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="n">
+        <v>1.21</v>
+      </c>
+    </row>
+    <row r="46" ht="55" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:31 UTC</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>AI Act | Shaping Europe’s digital future</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>https://digital-strategy.ec.europa.eu/en/policies/regulatory-framework-ai</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="n">
+        <v>2523</v>
+      </c>
+      <c r="I46" s="6" t="inlineStr">
+        <is>
+          <t>AI Act | Shaping Europe’s digital future Skip to main content AI Act The AI Act is the first-ever legal framework on AI, which addresses the risks of AI and positions Europe to play a leading role globally. The AI Act (Regulation (EU) 2024/1689 laying down harmonised rules on artificial intelligence</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="47" ht="55" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:31 UTC</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>https://www.frontiersin.org/articles/10.3389/frobt.2025.1563482/full</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not found</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="n">
+        <v>1.26</v>
+      </c>
+    </row>
+    <row r="48" ht="55" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:32 UTC</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>World Models: A Comprehensive Survey of Architectures, Methodologies, Reasoning Paradigms, and Applications</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2606.00133</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>PDF (arXiv abs-&gt;pdf rewrite (https://arxiv.org/abs/2606.00133))</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="n">
+        <v>19075</v>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>World Models: A Comprehensive Survey of Architectures, Methodologies, Reasoning Paradigms, and Applications Arif Hassan Zidan1, Yi Pan2, Hanqi Jiang2, Ruiyu Yan9, Wei Ruan2, Zihao Wu2, Lifeng Chen2, Weihang You2, Xinliang Li2, Bowen Chen3, Huawen Hu2, Peilong Wang10, Sizhuang Liu12, Jing Zhang5, Siy</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="49" ht="55" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:36 UTC</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>World Models: A Comprehensive Survey of Architectures, Methodologies, Reasoning Paradigms, and Applications</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2606.00133</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="n">
+        <v>19075</v>
+      </c>
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t>World Models: A Comprehensive Survey of Architectures, Methodologies, Reasoning Paradigms, and Applications Arif Hassan Zidan1, Yi Pan2, Hanqi Jiang2, Ruiyu Yan9, Wei Ruan2, Zihao Wu2, Lifeng Chen2, Weihang You2, Xinliang Li2, Bowen Chen3, Huawen Hu2, Peilong Wang10, Sizhuang Liu12, Jing Zhang5, Siy</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="n">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="50" ht="55" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>214</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mdpi.com/2073-431X/14/7/214</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>403</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="51" ht="55" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>ai research landscape 2026</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>https://adaline.ai/blog/ai-research-landscape-2026</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 500 Internal Server Error</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="52" ht="55" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:41 UTC</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>ai maturity model 2026</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>https://sema4.ai/resources/ai-maturity-model-2026</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>403</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="n">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="53" ht="55" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:41 UTC</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>ai inference economics framework investors</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>https://vistaequitypartners.com/insights/ai-inference-economics-framework-investors/</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>403</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="54" ht="55" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:41 UTC</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>artificial intelligence 2026</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>https://chambers.com/guides/artificial-intelligence-2026</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="n">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="55" ht="55" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:42 UTC</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>claude 3 7</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>https://www.anthropic.com/model-card/claude-3-7</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="n">
+        <v>6.62</v>
+      </c>
+    </row>
+    <row r="56" ht="55" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:48 UTC</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>agent computer interaction survey 2026</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>https://research.google/pubs/agent-computer-interaction-survey-2026/</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="57" ht="55" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:49 UTC</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>shaping the future of ai</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>https://www.weforum.org/publications/shaping-the-future-of-ai/</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>403</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="n">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="58" ht="55" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 21:20:49 UTC</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>full-source-test-24docs</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>open llm leaderboard 2026 analysis</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/blog/open-llm-leaderboard-2026-analysis</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="n">
+        <v>0.11</v>
       </c>
     </row>
   </sheetData>
@@ -2180,6 +3275,30 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>